<commit_message>
Add Palantir Technologies across all relevant analysis sheets
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Iran_War_Impact_Software_Internet_Analysis.xlsx
+++ b/Iran_War_Impact_Software_Internet_Analysis.xlsx
@@ -75,7 +75,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -89,11 +89,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -111,6 +139,8 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -476,7 +506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F33"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -493,11 +523,11 @@
           <t>IMPACT OF IRAN WAR ON SOFTWARE &amp; INTERNET — EXECUTIVE SUMMARY</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -537,11 +567,11 @@
           <t>DIGITAL ADVERTISING</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
+      <c r="B3" s="7" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="8" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -717,11 +747,11 @@
           <t>TRAVEL MARKETPLACES</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n"/>
-      <c r="C10" s="2" t="n"/>
-      <c r="D10" s="2" t="n"/>
-      <c r="E10" s="2" t="n"/>
-      <c r="F10" s="2" t="n"/>
+      <c r="B10" s="7" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="7" t="n"/>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -865,11 +895,11 @@
           <t>SOFTWARE &amp; INTERNET</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="B16" s="7" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1013,26 +1043,26 @@
           <t>CYBERSECURITY (BENEFICIARIES)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n"/>
-      <c r="C22" s="2" t="n"/>
-      <c r="D22" s="2" t="n"/>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="n"/>
+      <c r="B22" s="7" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="7" t="n"/>
+      <c r="E22" s="7" t="n"/>
+      <c r="F22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>CrowdStrike</t>
+          <t>Palantir Technologies</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Positive – Demand tailwind</t>
+          <t>Positive – Defense &amp; intelligence demand surge</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Q2 FY26 revenue $1.17B (+21% YoY); ARR $4.66B (+20% YoY)</t>
+          <t>FY2025 revenue $4.475B (+56% YoY); FY2026 guidance $7.18–7.20B (+61% YoY)</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -1042,19 +1072,19 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Record net new ARR of $221M; Iranian cyber threats boost enterprise security spend</t>
+          <t>Stock +85% in 2025; $10B US Army contract; Maven AI contract expanded to $1.275B; Israel MoD partnership since Oct 2024; Gov rev $2.4B (+53% YoY)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>CrowdStrike IR</t>
+          <t>Palantir Q4 2025 earnings; TradingView; Breaking Defense; Defense News</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Palo Alto Networks</t>
+          <t>CrowdStrike</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
@@ -1064,7 +1094,7 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Q2 FY26 revenue $2.6B (+15% YoY); FY26 guidance $11.28–11.31B (+22–23% YoY)</t>
+          <t>Q2 FY26 revenue $1.17B (+21% YoY); ARR $4.66B (+20% YoY)</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1074,210 +1104,242 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>NG Security ARR grew 33% YoY to $6.3B; acquired CyberArk for $25B</t>
+          <t>Record net new ARR of $221M; Iranian cyber threats boost enterprise security spend</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>CNBC; Palo Alto IR</t>
+          <t>CrowdStrike IR</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>Palo Alto Networks</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>Positive – Demand tailwind</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Q2 FY26 revenue $2.6B (+15% YoY); FY26 guidance $11.28–11.31B (+22–23% YoY)</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>2025–2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>NG Security ARR grew 33% YoY to $6.3B; acquired CyberArk for $25B</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>CNBC; Palo Alto IR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
           <t>Booz Allen Hamilton</t>
         </is>
       </c>
-      <c r="B25" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>Positive – Federal cyber demand</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>FY26 revenue guidance $12.0–12.5B; cyber revenue $2.5–2.8B (~23% of total)</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>2025–2026</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E26" s="4" t="inlineStr">
         <is>
           <t>8,000+ cyber professionals; 300 active projects; record $38B backlog</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F26" s="4" t="inlineStr">
         <is>
           <t>Booz Allen IR; GovConWire</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr"/>
-      <c r="D26" s="4" t="inlineStr"/>
-      <c r="E26" s="4" t="inlineStr"/>
-      <c r="F26" s="4" t="inlineStr"/>
-    </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr"/>
+      <c r="D27" s="4" t="inlineStr"/>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr">
         <is>
           <t>DEFENSE SECTOR (BENEFICIARIES)</t>
         </is>
       </c>
-      <c r="B27" s="2" t="n"/>
-      <c r="C27" s="2" t="n"/>
-      <c r="D27" s="2" t="n"/>
-      <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>RTX (Raytheon)</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>Positive – Stock surge</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>Stock +6.6% on Mar 2026 strikes; Q4 2025 revenue $24.24B (+12.1% YoY)</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>Mar 2026</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>FY26 EPS guidance $6.60–6.80 vs consensus $6.11</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>CNBC; Parameter.io</t>
-        </is>
-      </c>
+      <c r="B28" s="7" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="7" t="n"/>
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
+          <t>RTX (Raytheon)</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Positive – Stock surge</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Stock +6.6% on Mar 2026 strikes; Q4 2025 revenue $24.24B (+12.1% YoY)</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>FY26 EPS guidance $6.60–6.80 vs consensus $6.11</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>CNBC; Parameter.io</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
           <t>Lockheed Martin</t>
         </is>
       </c>
-      <c r="B29" s="6" t="inlineStr">
+      <c r="B30" s="6" t="inlineStr">
         <is>
           <t>Positive – Stock surge</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>Stock +6.9% on Mar 2026 strikes</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>Defense spending uplift from conflict escalation</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F30" s="4" t="inlineStr">
         <is>
           <t>CNBC Mar 2026</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr"/>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr"/>
-      <c r="D30" s="4" t="inlineStr"/>
-      <c r="E30" s="4" t="inlineStr"/>
-      <c r="F30" s="4" t="inlineStr"/>
-    </row>
     <row r="31">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="4" t="inlineStr"/>
+      <c r="C31" s="4" t="inlineStr"/>
+      <c r="D31" s="4" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr"/>
+      <c r="F31" s="4" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
         <is>
           <t>OIL &amp; MACRO IMPACT</t>
         </is>
       </c>
-      <c r="B31" s="2" t="n"/>
-      <c r="C31" s="2" t="n"/>
-      <c r="D31" s="2" t="n"/>
-      <c r="E31" s="2" t="n"/>
-      <c r="F31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Oil Prices → Consumer Spending → Ad Spend</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>Negative – Indirect</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Brent crude surged 15% ($67 → $81.40) during June 2025 escalation; US gas avg $3.13/gal</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Jun 2025</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>Strait of Hormuz carries 20% of global oil; higher energy costs compress consumer + ad spend</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Economist; Reuters</t>
-        </is>
-      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
+          <t>Oil Prices → Consumer Spending → Ad Spend</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Negative – Indirect</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Brent crude surged 15% ($67 → $81.40) during June 2025 escalation; US gas avg $3.13/gal</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Strait of Hormuz carries 20% of global oil; higher energy costs compress consumer + ad spend</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Economist; Reuters</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
           <t>S&amp;P 500 / Tech Stocks (Market)</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>Negative – Short-term, then recovery</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>S&amp;P 500 dropped ~0.7% on Jun 2025 strikes; historical avg drawdown 4.6% over 19 days</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D34" s="4" t="inlineStr">
         <is>
           <t>Historical pattern</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E34" s="4" t="inlineStr">
         <is>
           <t>Avg recovery to pre-event levels: 40 days (median 18 days); only 2 events caused &gt;20% crash</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F34" s="4" t="inlineStr">
         <is>
           <t>LPL Research; Yahoo Finance; Deutsche Bank</t>
         </is>
@@ -1322,13 +1384,13 @@
           <t>ADVERTISING MARKETPLACE COMPANIES — IRAN WAR REVENUE IMPACT &amp; EXPOSURE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -1657,13 +1719,13 @@
           <t>TRAVEL MARKETPLACE COMPANIES — IRAN WAR REVENUE IMPACT &amp; EXPOSURE</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
-      <c r="H1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="7" t="n"/>
+      <c r="H1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2015,7 +2077,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2033,12 +2095,12 @@
           <t>SOFTWARE &amp; INTERNET COMPANIES — IRAN WAR IMPACT ANALYSIS</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2302,17 +2364,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CrowdStrike</t>
+          <t>Palantir Technologies</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>$3.95B (FY2026 est)</t>
+          <t>$4.475B (FY2025)</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Demand surge from cyber threats</t>
+          <t>Major beneficiary — defense AI demand surge</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -2322,29 +2384,29 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Q2 FY26 revenue $1.17B (+21% YoY). ARR $4.66B (+20%). Record net new ARR $221M. Iranian cyber threats boost enterprise spending.</t>
+          <t>Stock soared 85% in 2025 driven by Iran-Israel conflict. Battlefield AI tools deployed via Israel MoD partnership (since Oct 2024). Maven Smart System contract expanded from $480M to $1.275B. $10B US Army contract signed Aug 2025. NATO adopted Maven AI for military planning. Permanent desk at US-led CMCC in southern Israel for Gaza operations. Gov revenue $2.402B (+53% YoY); US Gov revenue $1.855B (+55% YoY). US Commercial revenue surged 109% YoY to $1.465B as defense-adjacent enterprises adopted AI. CEO Karp: 'America has become more lethal, more confident' through Palantir tools.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>+$200M+ incremental ARR attributable to threat environment</t>
+          <t>FY2026 guidance $7.18–7.20B (+61% YoY) — 15% above consensus. Gov segment = 54% of revenue ($2.4B). Estimated $1B+ incremental revenue attributable to elevated defense/intelligence spending environment.</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>Geopolitical tensions are secular tailwind for cybersecurity</t>
+          <t>Iran-Israel conflict is a direct, cited driver of stock performance and contract pipeline. Forward P/E of 240x (10x sector median) reflects war premium. £1.5B UK defense deal (Sep 2025); $30M ICE contract. 954 customers in 2025; top-20 avg revenue $93.9M (up from $64.6M).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Palo Alto Networks</t>
+          <t>CrowdStrike</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>$9.15B (FY2025)</t>
+          <t>$3.95B (FY2026 est)</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -2359,34 +2421,34 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Q2 FY26 revenue $2.6B (+15% YoY). FY26 guidance $11.28–11.31B (+22–23%). NG Security ARR $6.3B (+33%).</t>
+          <t>Q2 FY26 revenue $1.17B (+21% YoY). ARR $4.66B (+20%). Record net new ARR $221M. Iranian cyber threats boost enterprise spending.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>+$500M+ incremental revenue from elevated threat demand</t>
+          <t>+$200M+ incremental ARR attributable to threat environment</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Acquired CyberArk ($25B) to expand security platform</t>
+          <t>Geopolitical tensions are secular tailwind for cybersecurity</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Booz Allen Hamilton</t>
+          <t>Palo Alto Networks</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>$11.4B (FY2025)</t>
+          <t>$9.15B (FY2025)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Federal cyber contract surge</t>
+          <t>Demand surge from cyber threats</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -2396,52 +2458,89 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>FY26 guidance $12.0–12.5B. Cyber revenue $2.5–2.8B (~23% of total). Record $38B backlog. 8,000+ cyber professionals.</t>
+          <t>Q2 FY26 revenue $2.6B (+15% YoY). FY26 guidance $11.28–11.31B (+22–23%). NG Security ARR $6.3B (+33%).</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>+$300M+ in cyber revenue growth</t>
+          <t>+$500M+ incremental revenue from elevated threat demand</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Leading federal cyber contractor; direct beneficiary of government response</t>
+          <t>Acquired CyberArk ($25B) to expand security platform</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>Booz Allen Hamilton</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>$11.4B (FY2025)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Federal cyber contract surge</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>FY26 guidance $12.0–12.5B. Cyber revenue $2.5–2.8B (~23% of total). Record $38B backlog. 8,000+ cyber professionals.</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>+$300M+ in cyber revenue growth</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Leading federal cyber contractor; direct beneficiary of government response</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>SentinelOne</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
         <is>
           <t>~$700M (FY2026 est)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Threat intelligence demand</t>
         </is>
       </c>
-      <c r="D12" s="6" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>Published Iran-specific threat intelligence briefs. Enterprise demand for Iranian APT detection capabilities increasing.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F13" s="4" t="inlineStr">
         <is>
           <t>Growth tailwind; exact amount undisclosed</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>Smaller player but growing share of Iranian threat detection market</t>
         </is>
@@ -2479,12 +2578,12 @@
           <t>HISTORICAL PRECEDENTS — GEOPOLITICAL CONFLICTS &amp; TECH/AD/TRAVEL SECTOR IMPACT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2759,7 +2858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2777,12 +2876,12 @@
           <t>QUANTIFIED REVENUE IMPACT SUMMARY — ALL SECTORS</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="7" t="n"/>
+      <c r="G1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -2836,12 +2935,12 @@
           <t>NEGATIVELY IMPACTED</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
+      <c r="B4" s="7" t="n"/>
+      <c r="C4" s="7" t="n"/>
+      <c r="D4" s="7" t="n"/>
+      <c r="E4" s="7" t="n"/>
+      <c r="F4" s="7" t="n"/>
+      <c r="G4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -3154,32 +3253,32 @@
           <t>POSITIVELY IMPACTED</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n"/>
-      <c r="C14" s="2" t="n"/>
-      <c r="D14" s="2" t="n"/>
-      <c r="E14" s="2" t="n"/>
-      <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="n"/>
+      <c r="B14" s="7" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="7" t="n"/>
+      <c r="E14" s="7" t="n"/>
+      <c r="F14" s="7" t="n"/>
+      <c r="G14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>CrowdStrike</t>
+          <t>Palantir Technologies</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>$3.95B</t>
+          <t>$4.475B (FY2025)</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>+$200M+ (threat-driven demand)</t>
+          <t>+$1B to +$1.5B (defense/intel demand)</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>+5%+</t>
+          <t>+22% to +33%</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -3189,29 +3288,29 @@
       </c>
       <c r="F15" s="4" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>Record ARR growth; Iranian APT activity drives enterprise security spend</t>
+          <t>Stock +85% in 2025 on Iran-Israel conflict. $10B Army contract, Maven expanded to $1.275B, Israel MoD partnership. Gov revenue grew 53% YoY. FY26 guidance $7.18–7.20B (+61% YoY) — 15% above consensus, reflecting sustained defense spending uplift.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Palo Alto Networks</t>
+          <t>CrowdStrike</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>$9.15B</t>
+          <t>$3.95B</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>+$500M+ (threat-driven demand)</t>
+          <t>+$200M+ (threat-driven demand)</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -3231,29 +3330,29 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>NG Security ARR grew 33%; $25B CyberArk acquisition strengthens position</t>
+          <t>Record ARR growth; Iranian APT activity drives enterprise security spend</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Booz Allen Hamilton</t>
+          <t>Palo Alto Networks</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>$11.4B</t>
+          <t>$9.15B</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>+$300M+ (federal cyber)</t>
+          <t>+$500M+ (threat-driven demand)</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>+3%+</t>
+          <t>+5%+</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -3268,29 +3367,29 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>Record $38B backlog; cyber revenue 23% of total and growing</t>
+          <t>NG Security ARR grew 33%; $25B CyberArk acquisition strengthens position</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>RTX (Raytheon)</t>
+          <t>Booz Allen Hamilton</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>$82B (FY2025)</t>
+          <t>$11.4B</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>+$2B to −$5B (defense orders)</t>
+          <t>+$300M+ (federal cyber)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>+2% to +6%</t>
+          <t>+3%+</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -3305,29 +3404,29 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Stock surged 6.6% on strikes; FY26 EPS guidance beat consensus by ~10%</t>
+          <t>Record $38B backlog; cyber revenue 23% of total and growing</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Lockheed Martin</t>
+          <t>RTX (Raytheon)</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>$71B (FY2025 est)</t>
+          <t>$82B (FY2025)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>+$1B to −$3B (defense orders)</t>
+          <t>+$2B to −$5B (defense orders)</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>+1% to +4%</t>
+          <t>+2% to +6%</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -3342,42 +3441,79 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>Stock surged 6.9% on strikes; increased international demand for defense systems</t>
+          <t>Stock surged 6.6% on strikes; FY26 EPS guidance beat consensus by ~10%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>Lockheed Martin</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>$71B (FY2025 est)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>+$1B to −$3B (defense orders)</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>+1% to +4%</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>Stock surged 6.9% on strikes; increased international demand for defense systems</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Oil &amp; Energy Sector</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>$2T+ (global)</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C21" s="4" t="inlineStr">
         <is>
           <t>+$50B to −$100B (price surge)</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>+2.5% to +5% (during spike)</t>
         </is>
       </c>
-      <c r="E20" s="6" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F21" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>Brent crude surged 15% during June 2025 escalation; Strait of Hormuz risk premium</t>
         </is>
@@ -3399,7 +3535,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3416,11 +3552,11 @@
           <t>CYBER WARFARE &amp; INFRASTRUCTURE RISK — IRAN CONFLICT</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="D1" s="2" t="n"/>
-      <c r="E1" s="2" t="n"/>
-      <c r="F1" s="2" t="n"/>
+      <c r="B1" s="7" t="n"/>
+      <c r="C1" s="7" t="n"/>
+      <c r="D1" s="7" t="n"/>
+      <c r="E1" s="7" t="n"/>
+      <c r="F1" s="8" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -3643,6 +3779,38 @@
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>Fortune; SentinelOne</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Palantir / Maven AI (US-Israel)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Defense &amp; Intelligence</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Battlefield AI, targeting, logistics coordination</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Palantir's Maven Smart System deployed across 5 combatant commands including CENTCOM. Provides automated target detection from satellite imagery and geolocation data. Permanent Palantir desk at US-led CMCC in southern Israel. NATO adopted Maven for military planning in 2025. Marine Corps signed enterprise license for Maven proliferation.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Palantir (primary); Pentagon; NATO; Israel MoD; US CENTCOM, EUCOM, INDOPACOM</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Breaking Defense; Defense News; DropSite News; Defense Scoop</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add cybersecurity segment exposure ranking with Iran attack timeline
Co-authored-by: ms4674 <ms4674@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Iran_War_Impact_Software_Internet_Analysis.xlsx
+++ b/Iran_War_Impact_Software_Internet_Analysis.xlsx
@@ -11,9 +11,10 @@
     <sheet name="Advertising Marketplaces" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Travel Marketplaces" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Software &amp; Internet" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Historical Precedents" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Revenue Impact Summary" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Cyber &amp; Infrastructure Risk" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cybersecurity Segments" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Historical Precedents" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Revenue Impact Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cyber &amp; Infrastructure Risk" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,8 +43,21 @@
     <font>
       <color rgb="00006100"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C55A11"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -72,6 +86,30 @@
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
         <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF4500"/>
+        <bgColor rgb="00FF4500"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFA500"/>
+        <bgColor rgb="00FFA500"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
+        <bgColor rgb="00FFD700"/>
       </patternFill>
     </fill>
   </fills>
@@ -121,7 +159,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -141,6 +179,28 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1179,11 +1239,11 @@
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr"/>
-      <c r="B27" s="4" t="inlineStr"/>
-      <c r="C27" s="4" t="inlineStr"/>
-      <c r="D27" s="4" t="inlineStr"/>
-      <c r="E27" s="4" t="inlineStr"/>
-      <c r="F27" s="4" t="inlineStr"/>
+      <c r="B27" s="7" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="7" t="n"/>
+      <c r="E27" s="7" t="n"/>
+      <c r="F27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr">
@@ -1263,11 +1323,11 @@
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr"/>
-      <c r="B31" s="4" t="inlineStr"/>
-      <c r="C31" s="4" t="inlineStr"/>
-      <c r="D31" s="4" t="inlineStr"/>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
+      <c r="B31" s="7" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="1" t="inlineStr">
@@ -2560,6 +2620,948 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>CYBERSECURITY SEGMENT EXPOSURE TO IRAN CONFLICT — RANKED BY GEOPOLITICAL DEMAND SENSITIVITY</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Cybersecurity Segment</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Market Size (2025–2026)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Growth Rate (CAGR)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Iran-Specific Threat Vector</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Demand Driver from Conflict</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Key Companies</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Government Spend Linkage</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>Evidence of Geopolitical Uplift</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>OT / ICS / SCADA Security</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>$4.64B (2025) → $9.37B (2030)</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>15.1%</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>BAUXITE / CyberAv3ngers (IRGC-linked) directly targeting Unitronics PLCs, fuel management systems, water utilities, and energy grids. 80–120 hacktivist groups active in Jun–Jul 2025.</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>HIGHEST: Iranian groups explicitly targeted US water utilities ($250K cost per incident), Israeli energy operators, and industrial control systems. Ransomware on OT surged 87% in 2025 and +49% in 2026. Attacks moved from device-level to mapping entire control loops.</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr">
+        <is>
+          <t>Dragos, Claroty ($3B valuation; $150M Series F in 2026), Nozomi Networks (acquired by Mitsubishi for ~$1B), Fortinet (OT appliances), Honeywell Forge</t>
+        </is>
+      </c>
+      <c r="G3" s="9" t="inlineStr">
+        <is>
+          <t>Pentagon cyber budget $15.1B (FY2026); CISA advisories on Iranian ICS threats (AA23-335a); 91% of orgs lack dedicated OT cyber resource — regulatory mandates expanding</t>
+        </is>
+      </c>
+      <c r="H3" s="9" t="inlineStr">
+        <is>
+          <t>Dragos 2026 report: OT threat groups surged; ransomware targeting OT up 87% then +49%. Iranian BAUXITE group capabilities progressing from PLCs to full control-loop mapping. Nozomi named Deloitte Fast 500. Claroty raised $150M and plans IPO.</t>
+        </is>
+      </c>
+      <c r="I3" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>$17B+ (2025 est)</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>~18–22%</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Iranian APTs (MuddyWater, Charming Kitten, BAUXITE) generating high-value intelligence. State-sponsored actors shifting to covert access accumulation in identity/cloud/edge systems.</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>VERY HIGH: 91% of security leaders plan to increase threat intel spending in 2026. 76% of orgs invest $250K+ annually. Iran APT tracking is a core use case driving subscription growth. Geopolitical conflict directly generates the 'product' (threat data) these companies sell.</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Recorded Future, Mandiant (Google Cloud), CrowdStrike Falcon Intelligence, SentinelOne (published Iran-specific briefs), Flashpoint</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>FBI/CISA joint advisories on Iranian threats; IC3 reports; Pentagon intelligence programs; Five Eyes sharing</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>Recorded Future: 91% of leaders increasing spend. SentinelOne published dedicated Iran outlook. Mandiant tracking multiple Iranian APT groups. 81% of orgs consolidating TI vendors in 2026. Conflict directly generates intelligence demand.</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>Defense / Government Cyber Platforms</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>$15.1B Pentagon cyber (FY2026); broader gov't $30B+</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>~4–10% (federal); higher for AI-defense</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>Direct military operations against Iran require battlefield AI, C4ISR, and cyber-kinetic coordination. Maven Smart System deployed across CENTCOM.</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>VERY HIGH: US-Israeli strikes on Iran (Feb–Mar 2026) triggered immediate demand for AI-driven targeting, intelligence fusion, and cyber offense/defense platforms. $10B Army contract to Palantir. Pentagon Maven expanded from $480M to $1.275B.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Palantir ($4.475B rev; +56% YoY), Booz Allen Hamilton ($11.4B; $2.5–2.8B cyber), Leidos, SAIC, General Dynamics IT, L3Harris</t>
+        </is>
+      </c>
+      <c r="G5" s="9" t="inlineStr">
+        <is>
+          <t>Pentagon cyber budget surged to $15.1B. FY2026 defense budget $961.6B. Iran explicitly named as threat in budget priorities alongside China, Russia, DPRK.</t>
+        </is>
+      </c>
+      <c r="H5" s="9" t="inlineStr">
+        <is>
+          <t>Palantir stock +85% in 2025; $10B Army deal; Maven AI adopted by NATO. Booz Allen record $38B backlog. Pentagon cyber budget +4% despite broader cuts.</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Cloud Security</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>$9.0B (2024) → $22.6B (2028)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>25.9%</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Iranian state actors shifting to targeting cloud environments, identity systems, and edge infrastructure. 400% spike in probing attacks on AWS post-strikes.</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>HIGH: Cloud workload protection surging as Iranian actors target cloud infrastructure. Google acquired Wiz for $32B. Organizations accelerating cloud security spend to harden ME-region data centers.</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>Zscaler ($3.31–3.32B FY26 guidance; +24%), Wiz (acquired for $32B), Palo Alto Prisma Cloud, CrowdStrike Falcon Cloud, Microsoft Defender for Cloud</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>AWS/Azure ME data centers (Bahrain, Qatar, UAE) under direct threat. Federal FedRAMP and StateRAMP requirements expanding.</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>Zscaler AI-Security pillar grew 80%+ YoY. Wiz $32B acquisition by Google — largest cybersecurity deal ever. 400% probing spike on AWS post Iran strikes.</t>
+        </is>
+      </c>
+      <c r="I6" s="11" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access Management (IAM)</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>$17.7B (2024) → $25.4B (2028)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>~10–15%</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Iranian actors focusing on identity system compromise as primary infiltration vector. 65% of breaches involve identity compromise.</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>HIGH: Enterprises allocating 10–15% of total cybersecurity budgets to IAM. Iranian APTs specifically targeting identity and credential stores for covert access.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>CyberArk (acquired by Palo Alto for $25B), Okta, SailPoint, Saviynt ($700M Series B), ID.me ($340M Series E), Microsoft Entra</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Federal zero-trust mandates (EO 14028) driving government IAM adoption. CISA emphasizes identity as foundational security layer.</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>CyberArk acquired for $25B by Palo Alto — reflects strategic value. Saviynt $700M funding round. IAM drew most VC capital in 2025. Recorded Future notes Iranian APTs specifically targeting identity systems.</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Endpoint Detection &amp; Response (EDR/XDR)</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>$12B+ (2025 est)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>~12–15%</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Iranian wiper malware (Fatimiyoun Electronic Team) designed to permanently destroy data. Endpoint protection is last line of defense against destructive payloads.</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>MODERATE-HIGH: Wiper malware is an Iranian speciality — EDR/XDR platforms must detect and block destructive payloads before execution. Enterprise refresh cycles accelerating.</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>CrowdStrike ($4.66B ARR; +20%), SentinelOne (~$700M), Microsoft Defender for Endpoint, Palo Alto Cortex XDR</t>
+        </is>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Federal CISA BOD 22-01 mandates EDR on government endpoints. Pentagon endpoint security contracts expanding.</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>CrowdStrike record ARR growth despite July 2024 outage. SentinelOne publishing Iran-specific detection content. Wiper malware specialization creates persistent demand signal.</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Managed Security Services (MSS/MDR)</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>$24.1B (2024) → $42.1B (2028)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>~15%</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Geopolitical supply-chain incidents intensify demand for 24/7 managed detection and response. SMEs lack in-house expertise to handle Iranian APT-level threats.</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>MODERATE: Mid-market and SME organizations lacking dedicated security teams are outsourcing monitoring in response to heightened threat advisories. Volume growth driver.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Secureworks, Arctic Wolf, Sophos MDR, AT&amp;T Cybersecurity, IBM Managed Security</t>
+        </is>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>CISA Shields Up advisories drive SME adoption of managed security. Government incentives for small critical infrastructure operators.</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>Geopolitical supply-chain incidents cited as MDR growth driver by Mordor Intelligence. 91% of orgs lack dedicated OT cyber resource — MDR fills the gap.</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Network Security / SASE</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>$25B+ (2025 est)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>~12–18%</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>DDoS attacks from Iranian proxy groups. Network-level filtering required to block state-sponsored scanning and botnet activity.</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>MODERATE: Fortinet Unified SASE billings grew 40% in Q4 2025. Network segmentation increasingly required to isolate OT from IT in critical infrastructure.</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>Fortinet ($6.80B; +14% YoY), Palo Alto SASE, Zscaler, Cisco, Juniper Networks (acquired by HPE)</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>Federal TIC 3.0 and zero-trust network access requirements. SASE adoption in government accelerating.</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>Fortinet SASE billings +40%; exceeded Rule of 45 for 6th consecutive year. Network security broadly benefits but less directly tied to Iran-specific vectors.</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>KEY FINDINGS — GEOPOLITICAL EXPOSURE RANKING</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+      <c r="F12" s="2" t="n"/>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Segment</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Rationale</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>#1 — MOST EXPOSED</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="13" t="inlineStr">
+        <is>
+          <t>OT / ICS / SCADA Security</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="15" t="inlineStr">
+        <is>
+          <t>Iranian IRGC-linked groups (BAUXITE, CyberAv3ngers) DIRECTLY and REPEATEDLY attacked US water utilities, Israeli energy, and industrial control systems in 2025. OT ransomware surged 87% then +49%. 91% of organizations lack dedicated OT security. Market doubling from $4.6B to $9.4B by 2030. This segment has the most direct, documented causal link between Iranian military action and demand.</t>
+        </is>
+      </c>
+      <c r="G14" s="14" t="n"/>
+      <c r="H14" s="14" t="n"/>
+      <c r="I14" s="14" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>#2 (tied)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="16" t="inlineStr">
+        <is>
+          <t>Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Iranian APT activity directly generates the intelligence product these companies sell. 91% of security leaders increasing spend. Conflict creates a self-reinforcing demand loop — more Iranian attacks → more intelligence needed → more subscriptions purchased.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>#2 (tied)</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>Defense / Government Cyber Platforms</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>Pentagon cyber budget hit $15.1B. Palantir's Maven AI deployed across CENTCOM for Iran operations. $10B Army contract. Iran explicitly named in defense budget priorities. This segment has the most direct GOVERNMENT BUDGET linkage to the conflict.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="n"/>
+      <c r="H16" s="2" t="n"/>
+      <c r="I16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>#4</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="16" t="inlineStr">
+        <is>
+          <t>Cloud Security</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>400% spike in probing attacks on AWS post-strikes. Iranian actors targeting cloud infrastructure. Google's $32B Wiz acquisition signals strategic importance. Growing but less directly tied to Iran than OT/TI.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>#5</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="16" t="inlineStr">
+        <is>
+          <t>Identity &amp; Access Management</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n"/>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>Iranian APTs specifically targeting identity stores for covert access. CyberArk acquired for $25B. High growth but driven by broader zero-trust trends beyond Iran.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>IRANIAN CYBER ATTACK TIMELINE — DRIVING OT/ICS AND THREAT INTEL DEMAND</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n"/>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
+      <c r="F20" s="2" t="n"/>
+      <c r="G20" s="2" t="n"/>
+      <c r="H20" s="2" t="n"/>
+      <c r="I20" s="2" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Attacker</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Method</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>Impact / Cost</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Segment Beneficiary</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Jun 2025</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>CyberAv3ngers (IRGC)</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>US Water Utilities (Texas)</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>PLC exploitation; default credentials; Unitronics devices</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>$250K per incident; service disruption; 3–12 hr recovery</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>OT/ICS Security (Dragos, Claroty, Nozomi)</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Jun–Jul 2025</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>80–120 hacktivist groups</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>US, Israel, Allied critical infrastructure</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Automated scanning; credential brute-force; wiper malware</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>Widespread reconnaissance; data leaks on Telegram/X</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>Threat Intelligence (Recorded Future, Mandiant)</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Jul 2025</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Homeland Justice (IRGC-linked)</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>Israeli Energy Operators</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Data breach; credential/config theft</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>$75K forensics cost; network diagrams exposed</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>OT/ICS Security; IAM</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Feb 28–Mar 1, 2026</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Cyber Islamic Resistance</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>US/Israeli Military Logistics</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>DoS; data-wiping attacks</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Operational disruption to logistics providers</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>Defense Cyber Platforms (Palantir, Booz Allen)</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Feb 28–Mar 1, 2026</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Handala Group</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Israeli Industrial Control Systems</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>ICS/SCADA targeting; manufacturing &amp; energy</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Claimed disruption of manufacturing and energy distribution</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>OT/ICS Security (Dragos, Claroty)</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Feb 28–Mar 1, 2026</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>Fatimiyoun Electronic Team</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>Western Financial &amp; Energy Firms</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>Wiper malware deployment</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Attempted permanent data destruction</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="n"/>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>EDR/XDR (CrowdStrike, SentinelOne)</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Mar 2026 (hours post-strike)</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>State-sponsored botnets</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>AWS Cloud Infrastructure</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>400% spike in probing/anomalous attacks</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Infrastructure hardening costs; potential service risk</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="n"/>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t>Cloud Security (Zscaler, Wiz, Palo Alto)</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="45">
+    <mergeCell ref="C16:E16"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="A12:I12"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="F24:G24"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="A20:I20"/>
+    <mergeCell ref="C13:E13"/>
+    <mergeCell ref="F23:G23"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="C15:E15"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="C14:E14"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="H26:I26"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2852,7 +3854,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3529,7 +4531,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>